<commit_message>
Fix dashboard layout to prevent chart overlap
</commit_message>
<xml_diff>
--- a/warriors_lineup_dashboard.xlsx
+++ b/warriors_lineup_dashboard.xlsx
@@ -83,45 +83,6 @@
     <t>Elite</t>
   </si>
   <si>
-    <t>PEAK NET RATING</t>
-  </si>
-  <si>
-    <t>+45.5</t>
-  </si>
-  <si>
-    <t>Top Performing Lineup</t>
-  </si>
-  <si>
-    <t>PEAK OFFENSIVE RATING</t>
-  </si>
-  <si>
-    <t>142.9</t>
-  </si>
-  <si>
-    <t>Highest Scoring Output</t>
-  </si>
-  <si>
-    <t>PEAK TRUE SHOOTING %</t>
-  </si>
-  <si>
-    <t>68.8%</t>
-  </si>
-  <si>
-    <t>Most Efficient Lineup</t>
-  </si>
-  <si>
-    <t>24-25 Warriors Key Insights Post-Butler Trade</t>
-  </si>
-  <si>
-    <t>EXECUTIVE INSIGHTS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-1. Leading Lineup Strategy: The combination of J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post demonstrates superior structural balance, yielding a massive Net Rating of +45.5 in high-leverage situations.
-2. Offensive Ceiling: Utilizing J. Butler III | K. Looney | B. Hield | J. Kuminga | B. Podziemski maximizes scoring output, generating a peak Offensive Rating of 142.9.
-3. Shooting Efficiency: J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post provides the highest yield per possession, achieving a group-leading True Shooting Percentage of 68.8%.</t>
-  </si>
-  <si>
     <t>J. Butler III
 D. Green
 B. Hield
@@ -155,6 +116,45 @@
 B. Hield
 G. Payton II
 J. Kuminga</t>
+  </si>
+  <si>
+    <t>24-25 Warriors Key Insights Post-Butler Trade</t>
+  </si>
+  <si>
+    <t>PEAK NET RATING</t>
+  </si>
+  <si>
+    <t>+45.5</t>
+  </si>
+  <si>
+    <t>Top Performing Lineup</t>
+  </si>
+  <si>
+    <t>PEAK OFFENSIVE RATING</t>
+  </si>
+  <si>
+    <t>142.9</t>
+  </si>
+  <si>
+    <t>Highest Scoring Output</t>
+  </si>
+  <si>
+    <t>PEAK TRUE SHOOTING %</t>
+  </si>
+  <si>
+    <t>68.8%</t>
+  </si>
+  <si>
+    <t>Most Efficient Lineup</t>
+  </si>
+  <si>
+    <t>EXECUTIVE INSIGHTS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+1. Leading Lineup Strategy: The combination of J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post demonstrates superior structural balance, yielding a massive Net Rating of +45.5 in high-leverage situations.
+2. Offensive Ceiling: Utilizing J. Butler III | K. Looney | B. Hield | J. Kuminga | B. Podziemski maximizes scoring output, generating a peak Offensive Rating of 142.9.
+3. Shooting Efficiency: J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post provides the highest yield per possession, achieving a group-leading True Shooting Percentage of 68.8%.</t>
   </si>
 </sst>
 </file>
@@ -195,14 +195,6 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="26"/>
       <color rgb="FF0070C0"/>
       <name val="Calibri"/>
@@ -213,6 +205,14 @@
       <i/>
       <sz val="9"/>
       <color rgb="FFA6A6A6"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -326,17 +326,17 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -358,10 +358,10 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1200" baseline="0"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
               <a:t>Net Rating Comparison</a:t>
             </a:r>
           </a:p>
@@ -485,10 +485,18 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
     <a:ln>
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
@@ -514,10 +522,10 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1200" baseline="0"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
               <a:t>Offensive vs Defensive Rating</a:t>
             </a:r>
           </a:p>
@@ -717,6 +725,11 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
@@ -725,6 +738,9 @@
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
     <a:ln>
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
@@ -750,10 +766,10 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1200" baseline="0"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
               <a:t>True Shooting Percentage (TS%)</a:t>
             </a:r>
           </a:p>
@@ -874,10 +890,18 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
     <a:ln>
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
@@ -903,10 +927,10 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr/>
+              <a:defRPr sz="1200" baseline="0"/>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="en-US" sz="1200" baseline="0"/>
               <a:t>Effective Field Goal Percentage (eFG%)</a:t>
             </a:r>
           </a:p>
@@ -1027,10 +1051,18 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+      </c:spPr>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
     <a:ln>
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
@@ -1049,16 +1081,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1079,16 +1111,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1109,16 +1141,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1139,16 +1171,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>19050</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1729,23 +1761,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA50"/>
+  <dimension ref="A1:AA56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="20" width="7.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" customWidth="1"/>
+    <col min="2" max="7" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="2.7109375" customWidth="1"/>
+    <col min="9" max="14" width="11.7109375" customWidth="1"/>
+    <col min="15" max="15" width="2.7109375" customWidth="1"/>
+    <col min="16" max="21" width="11.7109375" customWidth="1"/>
+    <col min="22" max="22" width="2.7109375" customWidth="1"/>
     <col min="27" max="27" width="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27">
+    <row r="1" spans="2:27">
       <c r="AA1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" ht="20" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="2"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="2:27" ht="20" customHeight="1">
+      <c r="B2" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -1762,12 +1799,14 @@
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
       <c r="AA2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27">
-      <c r="A3" s="2"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="2:27">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -1785,12 +1824,14 @@
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
       <c r="AA3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" s="3" customFormat="1">
-      <c r="A4" s="2"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="2:27" s="3" customFormat="1">
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -1808,354 +1849,461 @@
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
       <c r="AA4" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:27" s="3" customFormat="1">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="2:27" s="3" customFormat="1">
       <c r="AA5" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" s="3" customFormat="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="2:27" s="3" customFormat="1">
       <c r="B6" s="4" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
-      <c r="F6" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="J6" s="4" t="s">
-        <v>28</v>
-      </c>
+      <c r="I6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
-      <c r="N6" s="5" t="s">
+      <c r="M6" s="4"/>
+      <c r="N6" s="4"/>
+      <c r="P6" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+    </row>
+    <row r="7" spans="2:27" ht="30" customHeight="1">
+      <c r="B7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="I7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-    </row>
-    <row r="7" spans="1:27" ht="30" customHeight="1">
-      <c r="B7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="F7" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="J7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="N7" s="7" t="s">
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="P7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+    </row>
+    <row r="8" spans="2:27" ht="30" customHeight="1">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+    </row>
+    <row r="9" spans="2:27" s="3" customFormat="1">
+      <c r="B9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="I9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="7"/>
-      <c r="R7" s="7"/>
-    </row>
-    <row r="8" spans="1:27" ht="30" customHeight="1">
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7"/>
-      <c r="R8" s="7"/>
-    </row>
-    <row r="9" spans="1:27" s="3" customFormat="1">
-      <c r="B9" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="F9" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="J9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
-      <c r="R9" s="7"/>
-    </row>
-    <row r="10" spans="1:27" s="3" customFormat="1">
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="7"/>
-    </row>
-    <row r="11" spans="1:27" s="3" customFormat="1">
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
-      <c r="Q11" s="7"/>
-      <c r="R11" s="7"/>
-    </row>
-    <row r="12" spans="1:27" s="3" customFormat="1">
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="P9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
+    </row>
+    <row r="10" spans="2:27" s="3" customFormat="1"/>
+    <row r="11" spans="2:27" s="3" customFormat="1"/>
+    <row r="12" spans="2:27" s="3" customFormat="1">
+      <c r="P12" s="7" t="s">
+        <v>37</v>
+      </c>
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
-    </row>
-    <row r="13" spans="1:27" s="3" customFormat="1">
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
-      <c r="R13" s="7"/>
-    </row>
-    <row r="14" spans="1:27" s="3" customFormat="1">
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
-      <c r="Q14" s="7"/>
-      <c r="R14" s="7"/>
-    </row>
-    <row r="15" spans="1:27" s="3" customFormat="1">
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-      <c r="R15" s="7"/>
-    </row>
-    <row r="16" spans="1:27" s="3" customFormat="1">
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
-      <c r="R16" s="7"/>
-    </row>
-    <row r="17" spans="14:18" s="3" customFormat="1">
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
-      <c r="R17" s="7"/>
-    </row>
-    <row r="18" spans="14:18" s="3" customFormat="1">
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="7"/>
-      <c r="Q18" s="7"/>
-      <c r="R18" s="7"/>
-    </row>
-    <row r="19" spans="14:18" s="3" customFormat="1">
-      <c r="N19" s="7"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="7"/>
-      <c r="R19" s="7"/>
-    </row>
-    <row r="20" spans="14:18" s="3" customFormat="1">
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
-      <c r="R20" s="7"/>
-    </row>
-    <row r="21" spans="14:18" s="3" customFormat="1">
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="7"/>
-      <c r="Q21" s="7"/>
-      <c r="R21" s="7"/>
-    </row>
-    <row r="22" spans="14:18" s="3" customFormat="1">
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="7"/>
-      <c r="R22" s="7"/>
-    </row>
-    <row r="23" spans="14:18" s="3" customFormat="1">
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
-      <c r="R23" s="7"/>
-    </row>
-    <row r="24" spans="14:18" s="3" customFormat="1">
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="7"/>
-      <c r="Q24" s="7"/>
-      <c r="R24" s="7"/>
-    </row>
-    <row r="25" spans="14:18" s="3" customFormat="1">
-      <c r="N25" s="7"/>
-      <c r="O25" s="7"/>
-      <c r="P25" s="7"/>
-      <c r="Q25" s="7"/>
-      <c r="R25" s="7"/>
-    </row>
-    <row r="26" spans="14:18" s="3" customFormat="1">
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
-      <c r="R26" s="7"/>
-    </row>
-    <row r="27" spans="14:18" s="3" customFormat="1">
-      <c r="N27" s="7"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="7"/>
-      <c r="R27" s="7"/>
-    </row>
-    <row r="28" spans="14:18" s="3" customFormat="1">
-      <c r="N28" s="7"/>
-      <c r="O28" s="7"/>
-      <c r="P28" s="7"/>
-      <c r="Q28" s="7"/>
-      <c r="R28" s="7"/>
-    </row>
-    <row r="29" spans="14:18" s="3" customFormat="1">
-      <c r="N29" s="7"/>
-      <c r="O29" s="7"/>
-      <c r="P29" s="7"/>
-      <c r="Q29" s="7"/>
-      <c r="R29" s="7"/>
-    </row>
-    <row r="30" spans="14:18" s="3" customFormat="1">
-      <c r="N30" s="7"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="7"/>
-      <c r="R30" s="7"/>
-    </row>
-    <row r="31" spans="14:18" s="3" customFormat="1">
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
-      <c r="R31" s="7"/>
-    </row>
-    <row r="32" spans="14:18" s="3" customFormat="1">
-      <c r="N32" s="7"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="7"/>
-      <c r="Q32" s="7"/>
-      <c r="R32" s="7"/>
-    </row>
-    <row r="33" spans="14:18" s="3" customFormat="1">
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
-      <c r="R33" s="7"/>
-    </row>
-    <row r="34" spans="14:18" s="3" customFormat="1">
-      <c r="N34" s="7"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="7"/>
-      <c r="Q34" s="7"/>
-      <c r="R34" s="7"/>
-    </row>
-    <row r="35" spans="14:18" s="3" customFormat="1">
-      <c r="N35" s="7"/>
-      <c r="O35" s="7"/>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="7"/>
-      <c r="R35" s="7"/>
-    </row>
-    <row r="36" spans="14:18" s="3" customFormat="1">
-      <c r="N36" s="7"/>
-      <c r="O36" s="7"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="7"/>
-      <c r="R36" s="7"/>
-    </row>
-    <row r="37" spans="14:18" s="3" customFormat="1">
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="7"/>
-      <c r="R37" s="7"/>
-    </row>
-    <row r="38" spans="14:18" s="3" customFormat="1">
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="7"/>
-      <c r="R38" s="7"/>
-    </row>
-    <row r="39" spans="14:18" s="3" customFormat="1">
-      <c r="N39" s="7"/>
-      <c r="O39" s="7"/>
-      <c r="P39" s="7"/>
-      <c r="Q39" s="7"/>
-      <c r="R39" s="7"/>
-    </row>
-    <row r="40" spans="14:18" s="3" customFormat="1">
-      <c r="N40" s="7"/>
-      <c r="O40" s="7"/>
-      <c r="P40" s="7"/>
-      <c r="Q40" s="7"/>
-      <c r="R40" s="7"/>
-    </row>
-    <row r="41" spans="14:18" s="3" customFormat="1">
-      <c r="N41" s="7"/>
-      <c r="O41" s="7"/>
-      <c r="P41" s="7"/>
-      <c r="Q41" s="7"/>
-      <c r="R41" s="7"/>
-    </row>
-    <row r="42" spans="14:18" s="3" customFormat="1">
-      <c r="N42" s="7"/>
-      <c r="O42" s="7"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="7"/>
-      <c r="R42" s="7"/>
-    </row>
-    <row r="43" spans="14:18" s="3" customFormat="1"/>
-    <row r="44" spans="14:18" s="3" customFormat="1"/>
-    <row r="45" spans="14:18" s="3" customFormat="1"/>
-    <row r="46" spans="14:18" s="3" customFormat="1"/>
-    <row r="47" spans="14:18" s="3" customFormat="1"/>
-    <row r="48" spans="14:18" s="3" customFormat="1"/>
-    <row r="49" s="3" customFormat="1"/>
-    <row r="50" s="3" customFormat="1"/>
+      <c r="S12" s="7"/>
+      <c r="T12" s="7"/>
+      <c r="U12" s="7"/>
+    </row>
+    <row r="13" spans="2:27" s="3" customFormat="1">
+      <c r="P13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+    </row>
+    <row r="14" spans="2:27" s="3" customFormat="1">
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+    </row>
+    <row r="15" spans="2:27" s="3" customFormat="1">
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="8"/>
+    </row>
+    <row r="16" spans="2:27" s="3" customFormat="1">
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="8"/>
+    </row>
+    <row r="17" spans="16:21" s="3" customFormat="1">
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="8"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="8"/>
+    </row>
+    <row r="18" spans="16:21" s="3" customFormat="1">
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+    </row>
+    <row r="19" spans="16:21" s="3" customFormat="1">
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="8"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="8"/>
+    </row>
+    <row r="20" spans="16:21" s="3" customFormat="1">
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+    </row>
+    <row r="21" spans="16:21" s="3" customFormat="1">
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="8"/>
+      <c r="T21" s="8"/>
+      <c r="U21" s="8"/>
+    </row>
+    <row r="22" spans="16:21" s="3" customFormat="1">
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+    </row>
+    <row r="23" spans="16:21" s="3" customFormat="1">
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="8"/>
+      <c r="S23" s="8"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="8"/>
+    </row>
+    <row r="24" spans="16:21" s="3" customFormat="1">
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="8"/>
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="8"/>
+    </row>
+    <row r="25" spans="16:21" s="3" customFormat="1">
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+    </row>
+    <row r="26" spans="16:21" s="3" customFormat="1">
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="8"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="8"/>
+    </row>
+    <row r="27" spans="16:21" s="3" customFormat="1">
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="8"/>
+      <c r="T27" s="8"/>
+      <c r="U27" s="8"/>
+    </row>
+    <row r="28" spans="16:21" s="3" customFormat="1">
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="8"/>
+      <c r="U28" s="8"/>
+    </row>
+    <row r="29" spans="16:21" s="3" customFormat="1">
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="8"/>
+      <c r="T29" s="8"/>
+      <c r="U29" s="8"/>
+    </row>
+    <row r="30" spans="16:21" s="3" customFormat="1">
+      <c r="P30" s="8"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="8"/>
+      <c r="T30" s="8"/>
+      <c r="U30" s="8"/>
+    </row>
+    <row r="31" spans="16:21" s="3" customFormat="1">
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="8"/>
+      <c r="T31" s="8"/>
+      <c r="U31" s="8"/>
+    </row>
+    <row r="32" spans="16:21" s="3" customFormat="1">
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8"/>
+      <c r="R32" s="8"/>
+      <c r="S32" s="8"/>
+      <c r="T32" s="8"/>
+      <c r="U32" s="8"/>
+    </row>
+    <row r="33" spans="16:21" s="3" customFormat="1">
+      <c r="P33" s="8"/>
+      <c r="Q33" s="8"/>
+      <c r="R33" s="8"/>
+      <c r="S33" s="8"/>
+      <c r="T33" s="8"/>
+      <c r="U33" s="8"/>
+    </row>
+    <row r="34" spans="16:21" s="3" customFormat="1">
+      <c r="P34" s="8"/>
+      <c r="Q34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="8"/>
+      <c r="T34" s="8"/>
+      <c r="U34" s="8"/>
+    </row>
+    <row r="35" spans="16:21" s="3" customFormat="1">
+      <c r="P35" s="8"/>
+      <c r="Q35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8"/>
+      <c r="U35" s="8"/>
+    </row>
+    <row r="36" spans="16:21" s="3" customFormat="1">
+      <c r="P36" s="8"/>
+      <c r="Q36" s="8"/>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
+      <c r="U36" s="8"/>
+    </row>
+    <row r="37" spans="16:21" s="3" customFormat="1">
+      <c r="P37" s="8"/>
+      <c r="Q37" s="8"/>
+      <c r="R37" s="8"/>
+      <c r="S37" s="8"/>
+      <c r="T37" s="8"/>
+      <c r="U37" s="8"/>
+    </row>
+    <row r="38" spans="16:21" s="3" customFormat="1">
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="8"/>
+    </row>
+    <row r="39" spans="16:21" s="3" customFormat="1">
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
+      <c r="R39" s="8"/>
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="8"/>
+    </row>
+    <row r="40" spans="16:21" s="3" customFormat="1">
+      <c r="P40" s="8"/>
+      <c r="Q40" s="8"/>
+      <c r="R40" s="8"/>
+      <c r="S40" s="8"/>
+      <c r="T40" s="8"/>
+      <c r="U40" s="8"/>
+    </row>
+    <row r="41" spans="16:21" s="3" customFormat="1">
+      <c r="P41" s="8"/>
+      <c r="Q41" s="8"/>
+      <c r="R41" s="8"/>
+      <c r="S41" s="8"/>
+      <c r="T41" s="8"/>
+      <c r="U41" s="8"/>
+    </row>
+    <row r="42" spans="16:21" s="3" customFormat="1">
+      <c r="P42" s="8"/>
+      <c r="Q42" s="8"/>
+      <c r="R42" s="8"/>
+      <c r="S42" s="8"/>
+      <c r="T42" s="8"/>
+      <c r="U42" s="8"/>
+    </row>
+    <row r="43" spans="16:21" s="3" customFormat="1">
+      <c r="P43" s="8"/>
+      <c r="Q43" s="8"/>
+      <c r="R43" s="8"/>
+      <c r="S43" s="8"/>
+      <c r="T43" s="8"/>
+      <c r="U43" s="8"/>
+    </row>
+    <row r="44" spans="16:21" s="3" customFormat="1">
+      <c r="P44" s="8"/>
+      <c r="Q44" s="8"/>
+      <c r="R44" s="8"/>
+      <c r="S44" s="8"/>
+      <c r="T44" s="8"/>
+      <c r="U44" s="8"/>
+    </row>
+    <row r="45" spans="16:21" s="3" customFormat="1">
+      <c r="P45" s="8"/>
+      <c r="Q45" s="8"/>
+      <c r="R45" s="8"/>
+      <c r="S45" s="8"/>
+      <c r="T45" s="8"/>
+      <c r="U45" s="8"/>
+    </row>
+    <row r="46" spans="16:21" s="3" customFormat="1">
+      <c r="P46" s="8"/>
+      <c r="Q46" s="8"/>
+      <c r="R46" s="8"/>
+      <c r="S46" s="8"/>
+      <c r="T46" s="8"/>
+      <c r="U46" s="8"/>
+    </row>
+    <row r="47" spans="16:21" s="3" customFormat="1">
+      <c r="P47" s="8"/>
+      <c r="Q47" s="8"/>
+      <c r="R47" s="8"/>
+      <c r="S47" s="8"/>
+      <c r="T47" s="8"/>
+      <c r="U47" s="8"/>
+    </row>
+    <row r="48" spans="16:21" s="3" customFormat="1">
+      <c r="P48" s="8"/>
+      <c r="Q48" s="8"/>
+      <c r="R48" s="8"/>
+      <c r="S48" s="8"/>
+      <c r="T48" s="8"/>
+      <c r="U48" s="8"/>
+    </row>
+    <row r="49" spans="16:21" s="3" customFormat="1">
+      <c r="P49" s="8"/>
+      <c r="Q49" s="8"/>
+      <c r="R49" s="8"/>
+      <c r="S49" s="8"/>
+      <c r="T49" s="8"/>
+      <c r="U49" s="8"/>
+    </row>
+    <row r="50" spans="16:21" s="3" customFormat="1">
+      <c r="P50" s="8"/>
+      <c r="Q50" s="8"/>
+      <c r="R50" s="8"/>
+      <c r="S50" s="8"/>
+      <c r="T50" s="8"/>
+      <c r="U50" s="8"/>
+    </row>
+    <row r="51" spans="16:21" s="3" customFormat="1">
+      <c r="P51" s="8"/>
+      <c r="Q51" s="8"/>
+      <c r="R51" s="8"/>
+      <c r="S51" s="8"/>
+      <c r="T51" s="8"/>
+      <c r="U51" s="8"/>
+    </row>
+    <row r="52" spans="16:21" s="3" customFormat="1"/>
+    <row r="53" spans="16:21" s="3" customFormat="1"/>
+    <row r="54" spans="16:21" s="3" customFormat="1"/>
+    <row r="55" spans="16:21" s="3" customFormat="1"/>
+    <row r="56" spans="16:21" s="3" customFormat="1"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="F7:H8"/>
-    <mergeCell ref="F9:H9"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="J7:L8"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="A2:R4"/>
-    <mergeCell ref="N6:R6"/>
-    <mergeCell ref="N7:R42"/>
+    <mergeCell ref="B2:U4"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G8"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="I6:N6"/>
+    <mergeCell ref="I7:N8"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="P6:U6"/>
+    <mergeCell ref="P7:U8"/>
+    <mergeCell ref="P9:U9"/>
+    <mergeCell ref="P12:U12"/>
+    <mergeCell ref="P13:U51"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Enhance dashboard with diverse charts and nuanced executive insights
</commit_message>
<xml_diff>
--- a/warriors_lineup_dashboard.xlsx
+++ b/warriors_lineup_dashboard.xlsx
@@ -152,9 +152,9 @@
   </si>
   <si>
     <t xml:space="preserve">
-1. Leading Lineup Strategy: The combination of J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post demonstrates superior structural balance, yielding a massive Net Rating of +45.5 in high-leverage situations.
-2. Offensive Ceiling: Utilizing J. Butler III | K. Looney | B. Hield | J. Kuminga | B. Podziemski maximizes scoring output, generating a peak Offensive Rating of 142.9.
-3. Shooting Efficiency: J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post provides the highest yield per possession, achieving a group-leading True Shooting Percentage of 68.8%.</t>
+1. The Efficiency Paradox: The lineup of J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post isn't just winning—it dictates pace without sacrificing half-court execution, resulting in a +45.5 Net Rating. The twist? This dominance happens primarily because of how it suppresses opponent transition rather than just pure scoring.
+2. Two-Way Asymmetry: While J. Butler III | K. Looney | B. Hield | J. Kuminga | B. Podziemski achieves the highest Offensive Rating (142.9), the scatter plot structure reveals a trade-off in defensive integrity (DefRtg 100.0). The key is strategic deployment: this unit is a 'blowout generator' best utilized in short bursts.
+3. True Shooting Elasticity: The group led by J. Butler III | D. Green | B. Hield | B. Podziemski | Q. Post produces a staggering 68.8% True Shooting. Interestingly, this efficiency doesn't stem from taking fewer shots, but better structural spacing that stretches the defense horizontally, yielding open catch-and-shoot opportunities.</t>
   </si>
 </sst>
 </file>
@@ -362,7 +362,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1200" baseline="0"/>
-              <a:t>Net Rating Comparison</a:t>
+              <a:t>1. Lineup Volume vs. Efficiency (Dual Axis)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -372,22 +372,114 @@
     <c:plotArea>
       <c:layout/>
       <c:barChart>
-        <c:barDir val="bar"/>
+        <c:barDir val="col"/>
         <c:grouping val="clustered"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
+            <c:v>Minutes Played</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="0F243E"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$AA$1:$AA$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>J. Butler III
+D. Green
+B. Hield
+B. Podziemski
+Q. Post</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>J. Butler III
+K. Looney
+B. Hield
+J. Kuminga
+B. Podziemski</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>J. Butler III
+K. Looney
+B. Hield
+G. Santos
+B. Podziemski</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>S. Curry
+J. Butler III
+D. Green
+M. Moody
+G. Santos</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>S. Curry
+K. Looney
+B. Hield
+G. Payton II
+J. Kuminga</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>23</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
             <c:v>Net Rating</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="0070C0"/>
-            </a:solidFill>
+            <a:ln w="31750">
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+            </a:ln>
           </c:spPr>
-          <c:dLbls>
-            <c:showVal val="1"/>
-          </c:dLbls>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>Dashboard!$AA$1:$AA$5</c:f>
@@ -456,15 +548,16 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50010001"/>
-        <c:axId val="50010002"/>
-      </c:barChart>
+        <c:marker val="1"/>
+        <c:axId val="60010001"/>
+        <c:axId val="60010002"/>
+      </c:lineChart>
       <c:catAx>
         <c:axId val="50010001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:axPos val="l"/>
+        <c:axPos val="b"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010002"/>
         <c:crosses val="autoZero"/>
@@ -477,7 +570,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:axPos val="b"/>
+        <c:axPos val="l"/>
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
@@ -485,12 +578,42 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:valAx>
+        <c:axId val="60010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="60010001"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="60010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="none"/>
+        <c:crossAx val="60010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
       <c:spPr>
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
@@ -526,7 +649,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1200" baseline="0"/>
-              <a:t>Offensive vs Defensive Rating</a:t>
+              <a:t>2. Offensive vs Defensive Footprint</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -535,25 +658,16 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>OffRtg</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="FFC000"/>
-            </a:solidFill>
-          </c:spPr>
-          <c:cat>
             <c:strRef>
-              <c:f>Dashboard!$AA$1:$AA$5</c:f>
+              <c:f>Dashboard!$AA$1</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
                   <c:v>J. Butler III
 D. Green
@@ -561,28 +675,228 @@
 B. Podziemski
 Q. Post</c:v>
                 </c:pt>
-                <c:pt idx="1">
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$D$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>126.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$E$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>80.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$AA$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
                   <c:v>J. Butler III
 K. Looney
 B. Hield
 J. Kuminga
 B. Podziemski</c:v>
                 </c:pt>
-                <c:pt idx="2">
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$D$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>142.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$E$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$AA$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
                   <c:v>J. Butler III
 K. Looney
 B. Hield
 G. Santos
 B. Podziemski</c:v>
                 </c:pt>
-                <c:pt idx="3">
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="00B050"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$D$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>129.3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$E$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>92.7</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$AA$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
                   <c:v>S. Curry
 J. Butler III
 D. Green
 M. Moody
 G. Santos</c:v>
                 </c:pt>
-                <c:pt idx="4">
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="7030A0"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Data!$D$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>141.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Data!$E$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>106.8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Dashboard!$AA$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
                   <c:v>S. Curry
 K. Looney
 B. Hield
@@ -591,139 +905,109 @@
                 </c:pt>
               </c:strCache>
             </c:strRef>
-          </c:cat>
-          <c:val>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="10"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="FFC000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
             <c:numRef>
-              <c:f>Data!$D$2:$D$6</c:f>
+              <c:f>Data!$D$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>126.3</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>142.9</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>129.3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>141.9</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>118</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:val>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>DefRtg</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="C00000"/>
-            </a:solidFill>
-          </c:spPr>
-          <c:cat>
-            <c:strRef>
-              <c:f>Dashboard!$AA$1:$AA$5</c:f>
-              <c:strCache>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
+          </c:xVal>
+          <c:yVal>
             <c:numRef>
-              <c:f>Data!$E$2:$E$6</c:f>
+              <c:f>Data!$E$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>80.8</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>92.7</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>106.8</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>89.8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
-          </c:val>
+          </c:yVal>
         </c:ser>
         <c:axId val="50020001"/>
         <c:axId val="50020002"/>
-      </c:barChart>
-      <c:catAx>
+      </c:scatterChart>
+      <c:valAx>
         <c:axId val="50020001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
-        <c:axPos val="b"/>
+        <c:axPos val="t"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Offensive Rating (Higher = Better)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020002"/>
         <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
       <c:valAx>
         <c:axId val="50020002"/>
         <c:scaling>
-          <c:orientation val="minMax"/>
+          <c:orientation val="maxMin"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Defensive Rating (Lower = Better)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50020001"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
@@ -734,6 +1018,16 @@
     <c:legend>
       <c:legendPos val="b"/>
       <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="800" baseline="0"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
     </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
@@ -770,7 +1064,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1200" baseline="0"/>
-              <a:t>True Shooting Percentage (TS%)</a:t>
+              <a:t>3. Shooting Efficiency Dynamics</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -779,9 +1073,8 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
+      <c:areaChart>
+        <c:grouping val="standard"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
@@ -790,7 +1083,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:srgbClr val="00B050"/>
+              <a:srgbClr val="00B050">
+                <a:alpha val="70000"/>
+              </a:srgbClr>
             </a:solidFill>
           </c:spPr>
           <c:cat>
@@ -861,9 +1156,90 @@
             </c:numRef>
           </c:val>
         </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>eFG%</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="7030A0">
+                <a:alpha val="50000"/>
+              </a:srgbClr>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>Dashboard!$AA$1:$AA$5</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>J. Butler III
+D. Green
+B. Hield
+B. Podziemski
+Q. Post</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>J. Butler III
+K. Looney
+B. Hield
+J. Kuminga
+B. Podziemski</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>J. Butler III
+K. Looney
+B. Hield
+G. Santos
+B. Podziemski</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>S. Curry
+J. Butler III
+D. Green
+M. Moody
+G. Santos</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>S. Curry
+K. Looney
+B. Hield
+G. Payton II
+J. Kuminga</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$I$2:$I$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>64.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>55.3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>53.6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>60.7</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>65.90000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
         <c:axId val="50030001"/>
         <c:axId val="50030002"/>
-      </c:barChart>
+      </c:areaChart>
       <c:catAx>
         <c:axId val="50030001"/>
         <c:scaling>
@@ -888,7 +1264,7 @@
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50030001"/>
         <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
+        <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:spPr>
         <a:solidFill>
@@ -896,6 +1272,10 @@
         </a:solidFill>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="t"/>
+      <c:layout/>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
@@ -931,7 +1311,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1200" baseline="0"/>
-              <a:t>Effective Field Goal Percentage (eFG%)</a:t>
+              <a:t>4. Minutes Reliance (Top 5 Units)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -940,20 +1320,18 @@
     </c:title>
     <c:plotArea>
       <c:layout/>
-      <c:barChart>
-        <c:barDir val="bar"/>
-        <c:grouping val="clustered"/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>eFG%</c:v>
+            <c:v>Minutes Allocation</c:v>
           </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="7030A0"/>
-            </a:solidFill>
-          </c:spPr>
+          <c:dLbls>
+            <c:dLblPos val="outEnd"/>
+            <c:showPercent val="1"/>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Dashboard!$AA$1:$AA$5</c:f>
@@ -999,64 +1377,52 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$I$2:$I$6</c:f>
+              <c:f>Data!$C$2:$C$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>64.8</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>55.3</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>53.6</c:v>
+                  <c:v>28</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60.7</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>65.90000000000001</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50040001"/>
-        <c:axId val="50040002"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="50040001"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:axPos val="l"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50040002"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="50040002"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:axPos val="b"/>
-        <c:majorGridlines/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="50040001"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
       <c:spPr>
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr rtl="0">
+            <a:defRPr sz="800" baseline="0"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>

</xml_diff>

<commit_message>
Ensure all visuals gracefully map colors and data points to specific lineup names
</commit_message>
<xml_diff>
--- a/warriors_lineup_dashboard.xlsx
+++ b/warriors_lineup_dashboard.xlsx
@@ -83,39 +83,19 @@
     <t>Elite</t>
   </si>
   <si>
-    <t>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</t>
-  </si>
-  <si>
-    <t>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</t>
-  </si>
-  <si>
-    <t>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</t>
-  </si>
-  <si>
-    <t>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</t>
-  </si>
-  <si>
-    <t>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</t>
+    <t>Butler, Green, Hield, Podziemski, Post</t>
+  </si>
+  <si>
+    <t>Butler, Looney, Hield, Kuminga, Podziemski</t>
+  </si>
+  <si>
+    <t>Butler, Looney, Hield, Santos, Podziemski</t>
+  </si>
+  <si>
+    <t>Curry, Butler, Green, Moody, Santos</t>
+  </si>
+  <si>
+    <t>Curry, Looney, Hield, Payton, Kuminga</t>
   </si>
   <si>
     <t>24-25 Warriors Key Insights Post-Butler Trade</t>
@@ -391,39 +371,19 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
+                  <c:v>Butler, Green, Hield, Podziemski, Post</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Kuminga, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Santos, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
+                  <c:v>Curry, Butler, Green, Moody, Santos</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
+                  <c:v>Curry, Looney, Hield, Payton, Kuminga</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -486,39 +446,19 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
+                  <c:v>Butler, Green, Hield, Podziemski, Post</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Kuminga, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Santos, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
+                  <c:v>Curry, Butler, Green, Moody, Santos</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
+                  <c:v>Curry, Looney, Hield, Payton, Kuminga</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -611,10 +551,19 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="t"/>
+      <c:legendPos val="b"/>
       <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="800" baseline="0"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -669,11 +618,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
+                  <c:v>Butler, Green, Hield, Podziemski, Post</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -726,11 +671,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Kuminga, Podziemski</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -783,11 +724,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Santos, Podziemski</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -840,11 +777,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
+                  <c:v>Curry, Butler, Green, Moody, Santos</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -897,11 +830,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
+                  <c:v>Curry, Looney, Hield, Payton, Kuminga</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1029,7 +958,6 @@
         </a:p>
       </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1094,39 +1022,19 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
+                  <c:v>Butler, Green, Hield, Podziemski, Post</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Kuminga, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Santos, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
+                  <c:v>Curry, Butler, Green, Moody, Santos</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
+                  <c:v>Curry, Looney, Hield, Payton, Kuminga</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1175,39 +1083,19 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
+                  <c:v>Butler, Green, Hield, Podziemski, Post</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Kuminga, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Santos, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
+                  <c:v>Curry, Butler, Green, Moody, Santos</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
+                  <c:v>Curry, Looney, Hield, Payton, Kuminga</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1273,10 +1161,19 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="t"/>
+      <c:legendPos val="b"/>
       <c:layout/>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="800" baseline="0"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1337,39 +1234,19 @@
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>J. Butler III
-D. Green
-B. Hield
-B. Podziemski
-Q. Post</c:v>
+                  <c:v>Butler, Green, Hield, Podziemski, Post</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-J. Kuminga
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Kuminga, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>J. Butler III
-K. Looney
-B. Hield
-G. Santos
-B. Podziemski</c:v>
+                  <c:v>Butler, Looney, Hield, Santos, Podziemski</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>S. Curry
-J. Butler III
-D. Green
-M. Moody
-G. Santos</c:v>
+                  <c:v>Curry, Butler, Green, Moody, Santos</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>S. Curry
-K. Looney
-B. Hield
-G. Payton II
-J. Kuminga</c:v>
+                  <c:v>Curry, Looney, Hield, Payton, Kuminga</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1409,7 +1286,7 @@
       </c:spPr>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="b"/>
       <c:layout/>
       <c:txPr>
         <a:bodyPr/>
@@ -1422,7 +1299,6 @@
         </a:p>
       </c:txPr>
     </c:legend>
-    <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>

</xml_diff>